<commit_message>
Add cards-insights block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (8):
- blocks/cards-insights/cards-insights.css
- blocks/cards-insights/cards-insights.js
- tools/importer/import-why-firstnet.bundle.js
- tools/importer/import-why-firstnet.js
- tools/importer/page-templates.json
- tools/importer/parsers/cards-insights.js
- tools/importer/reports/import-why-firstnet.report.xlsx
- tools/importer/reports/why-firstnet.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-why-firstnet.report.xlsx
+++ b/tools/importer/reports/import-why-firstnet.report.xlsx
@@ -64,13 +64,13 @@
     <t>why-firstnet.report.json</t>
   </si>
   <si>
-    <t>["hero","columns-icons","cards","cards","columns","columns","accordion","form-newsletter"]</t>
+    <t>["hero","columns-icons","cards","cards-insights","columns","columns","accordion","form-newsletter"]</t>
   </si>
   <si>
     <t>why-firstnet</t>
   </si>
   <si>
-    <t>2026-02-11T16:10:15.754Z</t>
+    <t>2026-02-11T17:07:24.507Z</t>
   </si>
   <si>
     <t>Why Choose FirstNet for First Responder Communication Systems</t>

</xml_diff>